<commit_message>
idenfified wrong segment props initialization bug
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_24_11_10.xlsx
+++ b/simulations/scene/inputs/Scenarios_24_11_10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp45367\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp23692\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7937E954-3C86-445D-9E19-5F7F09E14CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A99BDFC-FDC9-4F97-A323-27A18616A78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28830" yWindow="-19695" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -14831,11 +14831,11 @@
       </c>
       <c r="L135" s="83"/>
       <c r="M135" s="83">
+        <f>0.0005 * 1.5</f>
+        <v>7.5000000000000002E-4</v>
+      </c>
+      <c r="N135" s="83">
         <f t="shared" ref="M135:W135" si="60">0.0005 / 10</f>
-        <v>5.0000000000000002E-5</v>
-      </c>
-      <c r="N135" s="83">
-        <f t="shared" si="60"/>
         <v>5.0000000000000002E-5</v>
       </c>
       <c r="O135" s="83">

</xml_diff>

<commit_message>
adjusted N parametrization to solve AA excess
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_24_11_10.xlsx
+++ b/simulations/scene/inputs/Scenarios_24_11_10.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp23692\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp16920\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4151DA82-33A1-43F4-BF38-7AB35356AC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC8005E-FC92-4DCF-8E4E-8FF6E48B0BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2488,7 +2488,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2696,6 +2696,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="11" fontId="16" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -23003,16 +23004,16 @@
         <v>5.0000000000000002E-11</v>
       </c>
       <c r="L221" s="83"/>
-      <c r="M221" s="83">
+      <c r="M221" s="101">
+        <f>0.00000000005 * 2</f>
+        <v>1E-10</v>
+      </c>
+      <c r="N221" s="101">
+        <f>0.00000000005 * 2</f>
+        <v>1E-10</v>
+      </c>
+      <c r="O221" s="83">
         <f t="shared" ref="M221:X221" si="71">0.00000000005 / 10 / 8</f>
-        <v>6.2500000000000006E-13</v>
-      </c>
-      <c r="N221" s="83">
-        <f t="shared" si="71"/>
-        <v>6.2500000000000006E-13</v>
-      </c>
-      <c r="O221" s="83">
-        <f t="shared" si="71"/>
         <v>6.2500000000000006E-13</v>
       </c>
       <c r="P221" s="83">
@@ -23095,16 +23096,14 @@
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="L222" s="83"/>
-      <c r="M222" s="83">
+      <c r="M222" s="101">
+        <v>0</v>
+      </c>
+      <c r="N222" s="101">
+        <v>1</v>
+      </c>
+      <c r="O222" s="83">
         <f t="shared" ref="M222:X222" si="72">0.0000001 / 2</f>
-        <v>4.9999999999999998E-8</v>
-      </c>
-      <c r="N222" s="83">
-        <f t="shared" si="72"/>
-        <v>4.9999999999999998E-8</v>
-      </c>
-      <c r="O222" s="83">
-        <f t="shared" si="72"/>
         <v>4.9999999999999998E-8</v>
       </c>
       <c r="P222" s="83">
@@ -23579,16 +23578,16 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="L227" s="99"/>
-      <c r="M227" s="99">
+      <c r="M227" s="101">
+        <f>0.00001 / 10</f>
+        <v>1.0000000000000002E-6</v>
+      </c>
+      <c r="N227" s="101">
+        <f>0.00001 / 10</f>
+        <v>1.0000000000000002E-6</v>
+      </c>
+      <c r="O227" s="99">
         <f t="shared" ref="M227:X227" si="76">0.00001 / 3</f>
-        <v>3.3333333333333337E-6</v>
-      </c>
-      <c r="N227" s="99">
-        <f t="shared" si="76"/>
-        <v>3.3333333333333337E-6</v>
-      </c>
-      <c r="O227" s="99">
-        <f t="shared" si="76"/>
         <v>3.3333333333333337E-6</v>
       </c>
       <c r="P227" s="99">
@@ -24128,13 +24127,13 @@
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="L233" s="83"/>
-      <c r="M233" s="83">
-        <f>0.00001 /2</f>
-        <v>5.0000000000000004E-6</v>
-      </c>
-      <c r="N233" s="83">
-        <f>0.00001 /2</f>
-        <v>5.0000000000000004E-6</v>
+      <c r="M233" s="101">
+        <f>0.00001 /2 / 10</f>
+        <v>5.0000000000000008E-7</v>
+      </c>
+      <c r="N233" s="101">
+        <f>0.00001 /2 / 10</f>
+        <v>5.0000000000000008E-7</v>
       </c>
       <c r="O233" s="83">
         <f t="shared" ref="O233:V233" si="79">0.00001 /2</f>
@@ -24191,7 +24190,7 @@
       </c>
       <c r="AC233" s="1" t="b">
         <f t="shared" si="66"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="234" spans="1:29" x14ac:dyDescent="0.25">
@@ -24230,16 +24229,16 @@
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="L234" s="83"/>
-      <c r="M234" s="83">
+      <c r="M234" s="101">
+        <f>0.000000005 / 5 / 100</f>
+        <v>1.0000000000000001E-11</v>
+      </c>
+      <c r="N234" s="101">
+        <f>0.000000005 / 5 / 100</f>
+        <v>1.0000000000000001E-11</v>
+      </c>
+      <c r="O234" s="83">
         <f t="shared" ref="M234:X234" si="80">0.000000005 / 5</f>
-        <v>1.0000000000000001E-9</v>
-      </c>
-      <c r="N234" s="83">
-        <f t="shared" si="80"/>
-        <v>1.0000000000000001E-9</v>
-      </c>
-      <c r="O234" s="83">
-        <f t="shared" si="80"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="P234" s="83">
@@ -24465,6 +24464,304 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G235:I236">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G236:AA236">
+    <cfRule type="colorScale" priority="363">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="364">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H129:AA130">
+    <cfRule type="colorScale" priority="365">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H212:AA212">
+    <cfRule type="colorScale" priority="367">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="366">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H213:AA213">
+    <cfRule type="colorScale" priority="369">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="368">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H214:AA214">
+    <cfRule type="colorScale" priority="370">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="371">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H215:AA215">
+    <cfRule type="colorScale" priority="373">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="372">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H216:AA216">
+    <cfRule type="colorScale" priority="375">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="374">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H217:AA217">
+    <cfRule type="colorScale" priority="377">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="376">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H220:AA220">
+    <cfRule type="colorScale" priority="379">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="378">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H223:AA223 H221:L222 O221:AA222">
+    <cfRule type="colorScale" priority="393">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="392">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H224:AA224">
+    <cfRule type="colorScale" priority="383">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="382">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H228:AA228">
+    <cfRule type="colorScale" priority="387">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="386">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H229:AA232 H233:L234 O233:AA234">
+    <cfRule type="colorScale" priority="389">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="388">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J235">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -24486,8 +24783,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G236:AA236">
-    <cfRule type="colorScale" priority="361">
+  <conditionalFormatting sqref="K235:L236">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24497,7 +24794,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="362">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24508,173 +24805,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H129:AA130">
-    <cfRule type="colorScale" priority="363">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H212:AA212">
-    <cfRule type="colorScale" priority="364">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="365">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H213:AA213">
-    <cfRule type="colorScale" priority="366">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="367">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H214:AA214">
-    <cfRule type="colorScale" priority="368">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="369">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H215:AA215">
-    <cfRule type="colorScale" priority="370">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="371">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H216:AA216">
-    <cfRule type="colorScale" priority="372">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="373">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H217:AA217">
-    <cfRule type="colorScale" priority="374">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="375">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H220:AA220">
-    <cfRule type="colorScale" priority="376">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="377">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H221:AA223">
+  <conditionalFormatting sqref="M235:AA236">
     <cfRule type="colorScale" priority="390">
       <colorScale>
         <cfvo type="min"/>
@@ -24696,29 +24827,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H224:AA224">
-    <cfRule type="colorScale" priority="380">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="381">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H228:AA228">
+  <conditionalFormatting sqref="AA225:AB225 AA226 H225:Z226">
     <cfRule type="colorScale" priority="384">
       <colorScale>
         <cfvo type="min"/>
@@ -24740,118 +24849,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H229:AA234">
-    <cfRule type="colorScale" priority="386">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="387">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J235">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K235:L236">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M235:AA236">
-    <cfRule type="colorScale" priority="388">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="389">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA225:AB225 AA226 H225:Z226">
-    <cfRule type="colorScale" priority="382">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="383">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AD129:AE130">
-    <cfRule type="colorScale" priority="51">
+    <cfRule type="colorScale" priority="53">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24863,7 +24862,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD131:AE131 H131:AB131">
-    <cfRule type="colorScale" priority="295">
+    <cfRule type="colorScale" priority="297">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24873,7 +24872,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="296">
+    <cfRule type="colorScale" priority="298">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24885,7 +24884,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD132:AE132 H132:AA132">
-    <cfRule type="colorScale" priority="299">
+    <cfRule type="colorScale" priority="301">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24895,7 +24894,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="300">
+    <cfRule type="colorScale" priority="302">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24907,7 +24906,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD134:AE134 H134:AB134">
-    <cfRule type="colorScale" priority="303">
+    <cfRule type="colorScale" priority="306">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24917,7 +24916,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="304">
+    <cfRule type="colorScale" priority="305">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24929,7 +24928,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD135:AE135 H135:AA135">
-    <cfRule type="colorScale" priority="307">
+    <cfRule type="colorScale" priority="310">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24939,7 +24938,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="308">
+    <cfRule type="colorScale" priority="309">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24951,7 +24950,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD140:AE140 H140:AB140">
-    <cfRule type="colorScale" priority="311">
+    <cfRule type="colorScale" priority="313">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24963,7 +24962,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD146:AE146 H146:AA146">
-    <cfRule type="colorScale" priority="313">
+    <cfRule type="colorScale" priority="315">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24973,7 +24972,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="314">
+    <cfRule type="colorScale" priority="316">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24983,7 +24982,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="315">
+    <cfRule type="colorScale" priority="317">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24995,7 +24994,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD162:AE162 H162:AA162">
-    <cfRule type="colorScale" priority="319">
+    <cfRule type="colorScale" priority="322">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25005,7 +25004,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="320">
+    <cfRule type="colorScale" priority="323">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25027,17 +25026,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD168:AE168 H168:AA168">
-    <cfRule type="colorScale" priority="325">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="326">
+    <cfRule type="colorScale" priority="328">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25048,6 +25037,16 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="327">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="329">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
debugged root growth model of Root_BRIDGES
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_24_11_10.xlsx
+++ b/simulations/scene/inputs/Scenarios_24_11_10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp16920\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC8005E-FC92-4DCF-8E4E-8FF6E48B0BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18BBDE0-1AF8-4D9A-AB75-86E63EC42322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2488,7 +2488,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2696,7 +2696,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="11" fontId="16" fillId="51" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -22904,15 +22903,15 @@
       </c>
       <c r="L220" s="83"/>
       <c r="M220" s="83">
-        <f t="shared" ref="M220:X220" si="70" xml:space="preserve"> 0.0000000000025</f>
-        <v>2.4999999999999998E-12</v>
+        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <v>2.4999999999999998E-11</v>
       </c>
       <c r="N220" s="83">
-        <f t="shared" si="70"/>
-        <v>2.4999999999999998E-12</v>
+        <f xml:space="preserve"> 0.0000000000025*10</f>
+        <v>2.4999999999999998E-11</v>
       </c>
       <c r="O220" s="83">
-        <f t="shared" si="70"/>
+        <f t="shared" ref="N220:X220" si="70" xml:space="preserve"> 0.0000000000025</f>
         <v>2.4999999999999998E-12</v>
       </c>
       <c r="P220" s="83">
@@ -22962,7 +22961,7 @@
       </c>
       <c r="AC220" s="1" t="b">
         <f t="shared" si="66"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221" spans="1:31" x14ac:dyDescent="0.25">
@@ -23004,16 +23003,16 @@
         <v>5.0000000000000002E-11</v>
       </c>
       <c r="L221" s="83"/>
-      <c r="M221" s="101">
-        <f>0.00000000005 * 2</f>
+      <c r="M221" s="83">
+        <f>0.00000000005 *2</f>
         <v>1E-10</v>
       </c>
-      <c r="N221" s="101">
-        <f>0.00000000005 * 2</f>
+      <c r="N221" s="83">
+        <f>0.00000000005 *2</f>
         <v>1E-10</v>
       </c>
       <c r="O221" s="83">
-        <f t="shared" ref="M221:X221" si="71">0.00000000005 / 10 / 8</f>
+        <f t="shared" ref="N221:X221" si="71">0.00000000005 / 10 / 8</f>
         <v>6.2500000000000006E-13</v>
       </c>
       <c r="P221" s="83">
@@ -23096,14 +23095,14 @@
         <v>4.9999999999999998E-7</v>
       </c>
       <c r="L222" s="83"/>
-      <c r="M222" s="101">
-        <v>0</v>
-      </c>
-      <c r="N222" s="101">
-        <v>1</v>
+      <c r="M222" s="83">
+        <v>0</v>
+      </c>
+      <c r="N222" s="83">
+        <v>0</v>
       </c>
       <c r="O222" s="83">
-        <f t="shared" ref="M222:X222" si="72">0.0000001 / 2</f>
+        <f t="shared" ref="N222:X222" si="72">0.0000001 / 2</f>
         <v>4.9999999999999998E-8</v>
       </c>
       <c r="P222" s="83">
@@ -23578,16 +23577,16 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="L227" s="99"/>
-      <c r="M227" s="101">
-        <f>0.00001 / 10</f>
-        <v>1.0000000000000002E-6</v>
-      </c>
-      <c r="N227" s="101">
-        <f>0.00001 / 10</f>
-        <v>1.0000000000000002E-6</v>
-      </c>
-      <c r="O227" s="99">
-        <f t="shared" ref="M227:X227" si="76">0.00001 / 3</f>
+      <c r="M227" s="83">
+        <f>0.00001 / 10 / 2 / 4</f>
+        <v>1.2500000000000002E-7</v>
+      </c>
+      <c r="N227" s="83">
+        <f>0.00001 / 10 / 2 / 4</f>
+        <v>1.2500000000000002E-7</v>
+      </c>
+      <c r="O227" s="83">
+        <f t="shared" ref="N227:X227" si="76">0.00001 / 3</f>
         <v>3.3333333333333337E-6</v>
       </c>
       <c r="P227" s="99">
@@ -24127,16 +24126,16 @@
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="L233" s="83"/>
-      <c r="M233" s="101">
-        <f>0.00001 /2 / 10</f>
-        <v>5.0000000000000008E-7</v>
-      </c>
-      <c r="N233" s="101">
-        <f>0.00001 /2 / 10</f>
-        <v>5.0000000000000008E-7</v>
+      <c r="M233" s="83">
+        <f>0.00001 /2</f>
+        <v>5.0000000000000004E-6</v>
+      </c>
+      <c r="N233" s="83">
+        <f t="shared" ref="N233:V233" si="79">0.00001 /2</f>
+        <v>5.0000000000000004E-6</v>
       </c>
       <c r="O233" s="83">
-        <f t="shared" ref="O233:V233" si="79">0.00001 /2</f>
+        <f t="shared" si="79"/>
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="P233" s="83">
@@ -24190,7 +24189,7 @@
       </c>
       <c r="AC233" s="1" t="b">
         <f t="shared" si="66"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234" spans="1:29" x14ac:dyDescent="0.25">
@@ -24229,16 +24228,16 @@
         <v>5.0000000000000004E-6</v>
       </c>
       <c r="L234" s="83"/>
-      <c r="M234" s="101">
-        <f>0.000000005 / 5 / 100</f>
-        <v>1.0000000000000001E-11</v>
-      </c>
-      <c r="N234" s="101">
-        <f>0.000000005 / 5 / 100</f>
-        <v>1.0000000000000001E-11</v>
+      <c r="M234" s="83">
+        <f t="shared" ref="M234:X234" si="80">0.000000005 / 5</f>
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="N234" s="83">
+        <f t="shared" si="80"/>
+        <v>1.0000000000000001E-9</v>
       </c>
       <c r="O234" s="83">
-        <f t="shared" ref="M234:X234" si="80">0.000000005 / 5</f>
+        <f t="shared" si="80"/>
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="P234" s="83">
@@ -24464,6 +24463,304 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G235:I236">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G236:AA236">
+    <cfRule type="colorScale" priority="366">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="365">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H129:AA130">
+    <cfRule type="colorScale" priority="367">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H212:AA212">
+    <cfRule type="colorScale" priority="369">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="368">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H213:AA213">
+    <cfRule type="colorScale" priority="371">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="370">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H214:AA214">
+    <cfRule type="colorScale" priority="372">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="373">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H215:AA215">
+    <cfRule type="colorScale" priority="374">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="375">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H216:AA216">
+    <cfRule type="colorScale" priority="377">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="376">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H217:AA217">
+    <cfRule type="colorScale" priority="379">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="378">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H220:AA220">
+    <cfRule type="colorScale" priority="381">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="380">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H221:AA223">
+    <cfRule type="colorScale" priority="394">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="395">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H224:AA224">
+    <cfRule type="colorScale" priority="385">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="384">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H228:AA228">
+    <cfRule type="colorScale" priority="388">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="389">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H229:AA234">
+    <cfRule type="colorScale" priority="391">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="390">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J235">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -24485,8 +24782,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G236:AA236">
-    <cfRule type="colorScale" priority="363">
+  <conditionalFormatting sqref="K235:L236">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24496,7 +24793,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="364">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24507,8 +24804,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H129:AA130">
-    <cfRule type="colorScale" priority="365">
+  <conditionalFormatting sqref="M227:O227">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24518,283 +24815,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H212:AA212">
-    <cfRule type="colorScale" priority="367">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="366">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H213:AA213">
-    <cfRule type="colorScale" priority="369">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="368">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H214:AA214">
-    <cfRule type="colorScale" priority="370">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="371">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H215:AA215">
-    <cfRule type="colorScale" priority="373">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="372">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H216:AA216">
-    <cfRule type="colorScale" priority="375">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="374">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H217:AA217">
-    <cfRule type="colorScale" priority="377">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="376">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H220:AA220">
-    <cfRule type="colorScale" priority="379">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="378">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H223:AA223 H221:L222 O221:AA222">
-    <cfRule type="colorScale" priority="393">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="392">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H224:AA224">
-    <cfRule type="colorScale" priority="383">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="382">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H228:AA228">
-    <cfRule type="colorScale" priority="387">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="386">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H229:AA232 H233:L234 O233:AA234">
-    <cfRule type="colorScale" priority="389">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="388">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J235">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K235:L236">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24806,7 +24827,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M235:AA236">
-    <cfRule type="colorScale" priority="390">
+    <cfRule type="colorScale" priority="392">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24816,7 +24837,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="391">
+    <cfRule type="colorScale" priority="393">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24828,7 +24849,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA225:AB225 AA226 H225:Z226">
-    <cfRule type="colorScale" priority="384">
+    <cfRule type="colorScale" priority="386">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24838,7 +24859,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="385">
+    <cfRule type="colorScale" priority="387">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24850,7 +24871,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD129:AE130">
-    <cfRule type="colorScale" priority="53">
+    <cfRule type="colorScale" priority="55">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24862,7 +24883,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD131:AE131 H131:AB131">
-    <cfRule type="colorScale" priority="297">
+    <cfRule type="colorScale" priority="299">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24872,7 +24893,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="298">
+    <cfRule type="colorScale" priority="300">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24884,7 +24905,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD132:AE132 H132:AA132">
-    <cfRule type="colorScale" priority="301">
+    <cfRule type="colorScale" priority="303">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24894,7 +24915,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="302">
+    <cfRule type="colorScale" priority="304">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24906,7 +24927,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD134:AE134 H134:AB134">
-    <cfRule type="colorScale" priority="306">
+    <cfRule type="colorScale" priority="308">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24916,7 +24937,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="305">
+    <cfRule type="colorScale" priority="307">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24928,7 +24949,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD135:AE135 H135:AA135">
-    <cfRule type="colorScale" priority="310">
+    <cfRule type="colorScale" priority="311">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24938,7 +24959,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="309">
+    <cfRule type="colorScale" priority="312">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24950,7 +24971,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD140:AE140 H140:AB140">
-    <cfRule type="colorScale" priority="313">
+    <cfRule type="colorScale" priority="315">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24962,7 +24983,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD146:AE146 H146:AA146">
-    <cfRule type="colorScale" priority="315">
+    <cfRule type="colorScale" priority="317">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24972,7 +24993,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="316">
+    <cfRule type="colorScale" priority="318">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24982,7 +25003,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="317">
+    <cfRule type="colorScale" priority="319">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -24994,7 +25015,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD162:AE162 H162:AA162">
-    <cfRule type="colorScale" priority="322">
+    <cfRule type="colorScale" priority="325">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25014,7 +25035,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="321">
+    <cfRule type="colorScale" priority="324">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25026,17 +25047,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD168:AE168 H168:AA168">
-    <cfRule type="colorScale" priority="328">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="327">
+    <cfRule type="colorScale" priority="330">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -25047,6 +25058,16 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="329">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="331">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>